<commit_message>
Kinda working ship Weird jittering with camera, may be because of fixed update ship controller stuff? Idk I'll figure it out later
</commit_message>
<xml_diff>
--- a/GunshipPrototype.xlsx
+++ b/GunshipPrototype.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benjamin Ellinger\Desktop\Digipen\DES315\Grading\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gary Yang\Documents\Programing\Unity\GunShip\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E2F2FA3-464F-4CDA-8098-B43D2F7947E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09B559AD-5786-41FC-AD9A-4D62F6C00099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements" sheetId="22" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
   <si>
     <t>POST-MORTEM (200+ Words)</t>
   </si>
@@ -1221,6 +1221,9 @@
   </si>
   <si>
     <t>Copy all gunship, weapon, boss, feedback, etc. code into this tab. Format it so that it is decently readable.</t>
+  </si>
+  <si>
+    <t>Full Credit</t>
   </si>
 </sst>
 </file>
@@ -2528,7 +2531,7 @@
     <row r="1" spans="1:5" s="3" customFormat="1" ht="23.4" thickBot="1">
       <c r="A1" s="18">
         <f>MIN(1,(MAX(D1,(SUM(A4:A963)+IF(ISBLANK(A2),0,MIN(0,A2-0.7))))))</f>
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="B1" s="32" t="s">
         <v>4</v>
@@ -2538,7 +2541,7 @@
       </c>
       <c r="D1" s="33">
         <f>MAX(A6,0)+MAX(A11,0)+MAX(A16,0)+MAX(A21,0)+MAX(A26,0)+MAX(A31,0)+COUNTIF(A7:A9,"&gt;0")*0.01+COUNTIF(A12:A14,"&gt;0")*0.01+COUNTIF(A17:A19,"&gt;0")*0.01+COUNTIF(A22:A24,"&gt;0")*0.01+COUNTIF(A27:A28,"&gt;0")*0.01+COUNTIF(A32:A34,"&gt;0")*0.01</f>
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="E1" s="9"/>
     </row>
@@ -2584,33 +2587,39 @@
       <c r="E6" s="11"/>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" ht="31.5" thickBot="1">
-      <c r="A7" s="34" t="str">
+      <c r="A7" s="34">
         <f>IF(LEFT(B7,2)="No",-0.1,IF(LEFT(B7,7)="Partial",0.01,IF(LEFT(B7,4)="Full",0.03,IF(LEFT(B7,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B7" s="35"/>
+        <v>0.03</v>
+      </c>
+      <c r="B7" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="C7" s="37" t="s">
         <v>21</v>
       </c>
       <c r="E7" s="12"/>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" ht="31.5" thickBot="1">
-      <c r="A8" s="34" t="str">
+      <c r="A8" s="34">
         <f>IF(LEFT(B8,2)="No",-0.1,IF(LEFT(B8,7)="Partial",0.01,IF(LEFT(B8,4)="Full",0.03,IF(LEFT(B8,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B8" s="35"/>
+        <v>0.03</v>
+      </c>
+      <c r="B8" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="C8" s="37" t="s">
         <v>20</v>
       </c>
       <c r="E8" s="12"/>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" ht="31.9" customHeight="1" thickBot="1">
-      <c r="A9" s="34" t="str">
+      <c r="A9" s="34">
         <f>IF(LEFT(B9,2)="No",-0.1,IF(LEFT(B9,7)="Partial",0.01,IF(LEFT(B9,4)="Full",0.03,IF(LEFT(B9,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B9" s="35"/>
+        <v>0.03</v>
+      </c>
+      <c r="B9" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="C9" s="37" t="s">
         <v>22</v>
       </c>
@@ -2653,11 +2662,13 @@
       <c r="E13" s="11"/>
     </row>
     <row r="14" spans="1:5" s="2" customFormat="1" ht="31.5" thickBot="1">
-      <c r="A14" s="34" t="str">
+      <c r="A14" s="34">
         <f>IF(LEFT(B14,2)="No",-0.1,IF(LEFT(B14,7)="Partial",0.01,IF(LEFT(B14,4)="Full",0.03,IF(LEFT(B14,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B14" s="35"/>
+        <v>0.03</v>
+      </c>
+      <c r="B14" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="C14" s="37" t="s">
         <v>28</v>
       </c>

</xml_diff>

<commit_message>
Ships Guns basic enemies
</commit_message>
<xml_diff>
--- a/GunshipPrototype.xlsx
+++ b/GunshipPrototype.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gary Yang\Documents\Programing\Unity\GunShip\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09B559AD-5786-41FC-AD9A-4D62F6C00099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39282E79-1DD0-4870-8F84-58CC544FE262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-78" yWindow="0" windowWidth="10032" windowHeight="13758" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements" sheetId="22" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="40">
   <si>
     <t>POST-MORTEM (200+ Words)</t>
   </si>
@@ -1224,6 +1224,9 @@
   </si>
   <si>
     <t>Full Credit</t>
+  </si>
+  <si>
+    <t>Partial Credit</t>
   </si>
 </sst>
 </file>
@@ -2531,7 +2534,7 @@
     <row r="1" spans="1:5" s="3" customFormat="1" ht="23.4" thickBot="1">
       <c r="A1" s="18">
         <f>MIN(1,(MAX(D1,(SUM(A4:A963)+IF(ISBLANK(A2),0,MIN(0,A2-0.7))))))</f>
-        <v>0.12</v>
+        <v>9.9999999999999992E-2</v>
       </c>
       <c r="B1" s="32" t="s">
         <v>4</v>
@@ -2664,10 +2667,10 @@
     <row r="14" spans="1:5" s="2" customFormat="1" ht="31.5" thickBot="1">
       <c r="A14" s="34">
         <f>IF(LEFT(B14,2)="No",-0.1,IF(LEFT(B14,7)="Partial",0.01,IF(LEFT(B14,4)="Full",0.03,IF(LEFT(B14,5)="Extra",0.05,"n/a"))))</f>
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C14" s="37" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
+ ship auto mode + ship hit effects + reworked explosions + reworked background generation + reworked enemy hit feedback
</commit_message>
<xml_diff>
--- a/GunshipPrototype.xlsx
+++ b/GunshipPrototype.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gary Yang\Documents\Programing\Unity\GunShip\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39282E79-1DD0-4870-8F84-58CC544FE262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE1E3F23-7D34-43ED-89E5-CAD9FC5E77A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-78" yWindow="0" windowWidth="10032" windowHeight="13758" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements" sheetId="22" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="42">
   <si>
     <t>POST-MORTEM (200+ Words)</t>
   </si>
@@ -1227,6 +1227,12 @@
   </si>
   <si>
     <t>Partial Credit</t>
+  </si>
+  <si>
+    <t>No Credit</t>
+  </si>
+  <si>
+    <t>This project went OK over all, I am finally getting the hang of organizing my self as well as  at least attempting to keep things organzied for as long as possible. I think the rate at which I try to change things means that this eventualy breaks down. I'm thinking I might need to add a step to my process where I refactor things instead of just plowing ahead. The problem, I think, is that when I'm trying to solve a problem my fixation is almost entirely blind to any other problems I'm creating by doing so. And this includes archetecture problems, it has in the past resulted me in making mega files because I just assumed I would need a function just here. Unity certainly isn't helping my habit by keeping all C# files ina  global space but I've forced myself by at least using folder based namespaces. Tweaking this project, things that had to scale.. enough I did get done but I also didn't get my full idea for this project in. My goal was to have it feel like you are in your ship going around a planet and that to be the point of reference to where you are in the world. There wasn't a good solution to this and in hindsight. this should have just been a flat world with a vertex warp of space. or just accept the difficulty of doing 2d planes around a sphere instead. But the more you know for next time. I did get to do some procedural work that I'm happy to say turned out better than I would have expected. The planet texture itself is a full perlin noise thing. And while I did want to add normal maps to it so it had some hight, some clouds.... etc.... by the time i realized i was wasting my time with an objective that way out paced the scope of what I was supposed to be doing at all, I had already gotten to the point that I was at. As I've talked without about this in length, I do know this is a problem, I'm trying to loop habits into making this better. But untill then... I'm sorry.</t>
   </si>
 </sst>
 </file>
@@ -2534,7 +2540,7 @@
     <row r="1" spans="1:5" s="3" customFormat="1" ht="23.4" thickBot="1">
       <c r="A1" s="18">
         <f>MIN(1,(MAX(D1,(SUM(A4:A963)+IF(ISBLANK(A2),0,MIN(0,A2-0.7))))))</f>
-        <v>9.9999999999999992E-2</v>
+        <v>0.11</v>
       </c>
       <c r="B1" s="32" t="s">
         <v>4</v>
@@ -2544,7 +2550,7 @@
       </c>
       <c r="D1" s="33">
         <f>MAX(A6,0)+MAX(A11,0)+MAX(A16,0)+MAX(A21,0)+MAX(A26,0)+MAX(A31,0)+COUNTIF(A7:A9,"&gt;0")*0.01+COUNTIF(A12:A14,"&gt;0")*0.01+COUNTIF(A17:A19,"&gt;0")*0.01+COUNTIF(A22:A24,"&gt;0")*0.01+COUNTIF(A27:A28,"&gt;0")*0.01+COUNTIF(A32:A34,"&gt;0")*0.01</f>
-        <v>0.04</v>
+        <v>0.11</v>
       </c>
       <c r="E1" s="9"/>
     </row>
@@ -2643,22 +2649,26 @@
       <c r="E11" s="12"/>
     </row>
     <row r="12" spans="1:5" s="2" customFormat="1" ht="31.9" customHeight="1" thickBot="1">
-      <c r="A12" s="34" t="str">
+      <c r="A12" s="34">
         <f>IF(LEFT(B12,2)="No",-0.1,IF(LEFT(B12,7)="Partial",0.01,IF(LEFT(B12,4)="Full",0.03,IF(LEFT(B12,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B12" s="35"/>
+        <v>0.03</v>
+      </c>
+      <c r="B12" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="C12" s="37" t="s">
         <v>23</v>
       </c>
       <c r="E12" s="12"/>
     </row>
     <row r="13" spans="1:5" s="2" customFormat="1" ht="31.5" thickBot="1">
-      <c r="A13" s="34" t="str">
+      <c r="A13" s="34">
         <f>IF(LEFT(B13,2)="No",-0.1,IF(LEFT(B13,7)="Partial",0.01,IF(LEFT(B13,4)="Full",0.03,IF(LEFT(B13,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B13" s="35"/>
+        <v>0.03</v>
+      </c>
+      <c r="B13" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="C13" s="37" t="s">
         <v>24</v>
       </c>
@@ -2667,10 +2677,10 @@
     <row r="14" spans="1:5" s="2" customFormat="1" ht="31.5" thickBot="1">
       <c r="A14" s="34">
         <f>IF(LEFT(B14,2)="No",-0.1,IF(LEFT(B14,7)="Partial",0.01,IF(LEFT(B14,4)="Full",0.03,IF(LEFT(B14,5)="Extra",0.05,"n/a"))))</f>
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C14" s="37" t="s">
         <v>28</v>
@@ -2692,33 +2702,39 @@
       <c r="E16" s="12"/>
     </row>
     <row r="17" spans="1:5" s="2" customFormat="1" ht="31.5" thickBot="1">
-      <c r="A17" s="34" t="str">
+      <c r="A17" s="34">
         <f>IF(LEFT(B17,2)="No",-0.1,IF(LEFT(B17,7)="Partial",0.01,IF(LEFT(B17,4)="Full",0.03,IF(LEFT(B17,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B17" s="35"/>
+        <v>0.03</v>
+      </c>
+      <c r="B17" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="C17" s="37" t="s">
         <v>25</v>
       </c>
       <c r="E17" s="12"/>
     </row>
     <row r="18" spans="1:5" s="2" customFormat="1" ht="31.9" customHeight="1" thickBot="1">
-      <c r="A18" s="34" t="str">
+      <c r="A18" s="34">
         <f>IF(LEFT(B18,2)="No",-0.1,IF(LEFT(B18,7)="Partial",0.01,IF(LEFT(B18,4)="Full",0.03,IF(LEFT(B18,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B18" s="35"/>
+        <v>0.01</v>
+      </c>
+      <c r="B18" s="35" t="s">
+        <v>39</v>
+      </c>
       <c r="C18" s="37" t="s">
         <v>26</v>
       </c>
       <c r="E18" s="11"/>
     </row>
     <row r="19" spans="1:5" s="2" customFormat="1" ht="31.5" thickBot="1">
-      <c r="A19" s="34" t="str">
+      <c r="A19" s="34">
         <f>IF(LEFT(B19,2)="No",-0.1,IF(LEFT(B19,7)="Partial",0.01,IF(LEFT(B19,4)="Full",0.03,IF(LEFT(B19,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B19" s="35"/>
+        <v>0.03</v>
+      </c>
+      <c r="B19" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="C19" s="37" t="s">
         <v>18</v>
       </c>
@@ -2739,33 +2755,39 @@
       <c r="E21" s="11"/>
     </row>
     <row r="22" spans="1:5" s="2" customFormat="1" ht="31.5" thickBot="1">
-      <c r="A22" s="34" t="str">
+      <c r="A22" s="34">
         <f>IF(LEFT(B22,2)="No",-0.1,IF(LEFT(B22,7)="Partial",0.01,IF(LEFT(B22,4)="Full",0.03,IF(LEFT(B22,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B22" s="35"/>
+        <v>-0.1</v>
+      </c>
+      <c r="B22" s="35" t="s">
+        <v>40</v>
+      </c>
       <c r="C22" s="37" t="s">
         <v>19</v>
       </c>
       <c r="E22" s="40"/>
     </row>
     <row r="23" spans="1:5" s="2" customFormat="1" ht="31.9" customHeight="1" thickBot="1">
-      <c r="A23" s="34" t="str">
+      <c r="A23" s="34">
         <f>IF(LEFT(B23,2)="No",-0.1,IF(LEFT(B23,7)="Partial",0.01,IF(LEFT(B23,4)="Full",0.03,IF(LEFT(B23,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B23" s="35"/>
+        <v>0.01</v>
+      </c>
+      <c r="B23" s="35" t="s">
+        <v>39</v>
+      </c>
       <c r="C23" s="5" t="s">
         <v>17</v>
       </c>
       <c r="E23" s="12"/>
     </row>
     <row r="24" spans="1:5" s="2" customFormat="1" ht="31.5" thickBot="1">
-      <c r="A24" s="34" t="str">
+      <c r="A24" s="34">
         <f>IF(LEFT(B24,2)="No",-0.1,IF(LEFT(B24,7)="Partial",0.01,IF(LEFT(B24,4)="Full",0.03,IF(LEFT(B24,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B24" s="35"/>
+        <v>0.03</v>
+      </c>
+      <c r="B24" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="C24" s="37" t="s">
         <v>27</v>
       </c>
@@ -2786,11 +2808,13 @@
       <c r="E26" s="12"/>
     </row>
     <row r="27" spans="1:5" s="2" customFormat="1" ht="31.9" customHeight="1" thickBot="1">
-      <c r="A27" s="34" t="str">
+      <c r="A27" s="34">
         <f>IF(LEFT(B27,2)="No",-0.1,IF(LEFT(B27,7)="Partial",0.01,IF(LEFT(B27,4)="Full",0.03,IF(LEFT(B27,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B27" s="35"/>
+        <v>-0.1</v>
+      </c>
+      <c r="B27" s="35" t="s">
+        <v>40</v>
+      </c>
       <c r="C27" s="37" t="s">
         <v>15</v>
       </c>
@@ -3193,11 +3217,13 @@
     <row r="2" spans="1:1" s="7" customFormat="1" ht="15.9" thickBot="1">
       <c r="A2" s="8" t="str">
         <f>IF(LEN(A3) &gt; 2000,"-----",IF(LEN(A3) &gt; 1000,"---",IF(LEN(A3) &gt; 500,"You need more post-mortem reflection.",IF(A3&gt;0,"You need A LOT MORE post-mortem reflection.","How did the project go? What did you learn? What could you improve?"))))</f>
-        <v>How did the project go? What did you learn? What could you improve?</v>
+        <v>---</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="409.5" customHeight="1">
-      <c r="A3" s="48"/>
+      <c r="A3" s="48" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="49"/>

</xml_diff>